<commit_message>
feat: Add professional Excel formatting based on BCI/Northleaf analysis
Updated generate_templates.py with institutional-quality formatting:
- Navy blue headers (#01395D) matching BCI case study
- Quartile color coding (red→yellow→light green→green)
- Scenario coloring (Bear=red, Base=blue, Bull=green)
- Professional number formatting with borders

New templates added:
- 16_precedent_transactions.xlsx
- 19_value_creation_waterfall.xlsx (MOIC + IRR bridges)
- 22_sensitivity_table.xlsx (Entry vs Exit matrix)
- 23_debt_schedule.xlsx (with credit metrics)
- 25_returns_analysis.xlsx (Gross/Net with fee waterfall)
- 27_deal_showcase.xlsx
- 28_cost_of_capital.xlsx

All 19 templates regenerated with consistent professional styling.

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/ii_skills/shared/excel_templates/05_time_series.xlsx
+++ b/src/ii_skills/shared/excel_templates/05_time_series.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,10 +29,21 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="0001395D"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
     <font>
       <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -44,8 +55,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004A4A4A"/>
-        <bgColor rgb="004A4A4A"/>
+        <fgColor rgb="0001395D"/>
+        <bgColor rgb="0001395D"/>
       </patternFill>
     </fill>
   </fills>
@@ -61,13 +72,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -157,7 +170,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Performance Comparison</a:t>
+              <a:t>Price Performance (Indexed)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -171,7 +184,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Time_Series'!B1</f>
+              <f>'Time_Series'!C5</f>
             </strRef>
           </tx>
           <spPr>
@@ -189,12 +202,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Time_Series'!$A$2:$A$13</f>
+              <f>'Time_Series'!$B$6:$B$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Time_Series'!$B$2:$B$13</f>
+              <f>'Time_Series'!$C$6:$C$17</f>
             </numRef>
           </val>
         </ser>
@@ -203,7 +216,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Time_Series'!C1</f>
+              <f>'Time_Series'!D5</f>
             </strRef>
           </tx>
           <spPr>
@@ -221,12 +234,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Time_Series'!$A$2:$A$13</f>
+              <f>'Time_Series'!$B$6:$B$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Time_Series'!$C$2:$C$13</f>
+              <f>'Time_Series'!$D$6:$D$17</f>
             </numRef>
           </val>
         </ser>
@@ -235,7 +248,7 @@
           <order val="2"/>
           <tx>
             <strRef>
-              <f>'Time_Series'!D1</f>
+              <f>'Time_Series'!E5</f>
             </strRef>
           </tx>
           <spPr>
@@ -253,12 +266,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Time_Series'!$A$2:$A$13</f>
+              <f>'Time_Series'!$B$6:$B$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Time_Series'!$D$2:$D$13</f>
+              <f>'Time_Series'!$E$6:$E$17</f>
             </numRef>
           </val>
         </ser>
@@ -307,7 +320,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Indexed Value</a:t>
+                  <a:t>Index</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -331,12 +344,12 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>5</col>
+      <col>6</col>
       <colOff>0</colOff>
-      <row>1</row>
+      <row>4</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5400000" cy="2700000"/>
+    <ext cx="5400000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -643,251 +656,275 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1"/>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Share Price Performance</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Indexed to 100 at start date</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
+    <row r="5">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Subject</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Benchmark_1</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Benchmark_2</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Benchmark 1</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Benchmark 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="4" t="n">
         <v>45292</v>
       </c>
-      <c r="B2" t="n">
+      <c r="C6" t="n">
         <v>100</v>
       </c>
-      <c r="C2" t="n">
+      <c r="D6" t="n">
         <v>100</v>
       </c>
-      <c r="D2" t="n">
+      <c r="E6" t="n">
         <v>100</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
+    <row r="7">
+      <c r="B7" s="4" t="n">
         <v>45322</v>
       </c>
-      <c r="B3" t="n">
+      <c r="C7" t="n">
         <v>105.2</v>
       </c>
-      <c r="C3" t="n">
+      <c r="D7" t="n">
         <v>102.8</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E7" t="n">
         <v>101.5</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
+    <row r="8">
+      <c r="B8" s="4" t="n">
         <v>45352</v>
       </c>
-      <c r="B4" t="n">
+      <c r="C8" t="n">
         <v>108.7</v>
       </c>
-      <c r="C4" t="n">
+      <c r="D8" t="n">
         <v>104.2</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E8" t="n">
         <v>103.8</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
+    <row r="9">
+      <c r="B9" s="4" t="n">
         <v>45382</v>
       </c>
-      <c r="B5" t="n">
+      <c r="C9" t="n">
         <v>112.3</v>
       </c>
-      <c r="C5" t="n">
+      <c r="D9" t="n">
         <v>107.5</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E9" t="n">
         <v>106.2</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
+    <row r="10">
+      <c r="B10" s="4" t="n">
         <v>45412</v>
       </c>
-      <c r="B6" t="n">
+      <c r="C10" t="n">
         <v>118.5</v>
       </c>
-      <c r="C6" t="n">
+      <c r="D10" t="n">
         <v>110.2</v>
       </c>
-      <c r="D6" t="n">
+      <c r="E10" t="n">
         <v>108.5</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
+    <row r="11">
+      <c r="B11" s="4" t="n">
         <v>45442</v>
       </c>
-      <c r="B7" t="n">
+      <c r="C11" t="n">
         <v>115.2</v>
       </c>
-      <c r="C7" t="n">
+      <c r="D11" t="n">
         <v>108.5</v>
       </c>
-      <c r="D7" t="n">
+      <c r="E11" t="n">
         <v>107.2</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
+    <row r="12">
+      <c r="B12" s="4" t="n">
         <v>45472</v>
       </c>
-      <c r="B8" t="n">
+      <c r="C12" t="n">
         <v>122.8</v>
       </c>
-      <c r="C8" t="n">
+      <c r="D12" t="n">
         <v>112.3</v>
       </c>
-      <c r="D8" t="n">
+      <c r="E12" t="n">
         <v>110.5</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
+    <row r="13">
+      <c r="B13" s="4" t="n">
         <v>45502</v>
       </c>
-      <c r="B9" t="n">
+      <c r="C13" t="n">
         <v>128.5</v>
       </c>
-      <c r="C9" t="n">
+      <c r="D13" t="n">
         <v>115.8</v>
       </c>
-      <c r="D9" t="n">
+      <c r="E13" t="n">
         <v>113.2</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="n">
+    <row r="14">
+      <c r="B14" s="4" t="n">
         <v>45532</v>
       </c>
-      <c r="B10" t="n">
+      <c r="C14" t="n">
         <v>135.2</v>
       </c>
-      <c r="C10" t="n">
+      <c r="D14" t="n">
         <v>118.2</v>
       </c>
-      <c r="D10" t="n">
+      <c r="E14" t="n">
         <v>116.8</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
+    <row r="15">
+      <c r="B15" s="4" t="n">
         <v>45562</v>
       </c>
-      <c r="B11" t="n">
+      <c r="C15" t="n">
         <v>142.1</v>
       </c>
-      <c r="C11" t="n">
+      <c r="D15" t="n">
         <v>122.5</v>
       </c>
-      <c r="D11" t="n">
+      <c r="E15" t="n">
         <v>119.5</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
+    <row r="16">
+      <c r="B16" s="4" t="n">
         <v>45592</v>
       </c>
-      <c r="B12" t="n">
+      <c r="C16" t="n">
         <v>138.5</v>
       </c>
-      <c r="C12" t="n">
+      <c r="D16" t="n">
         <v>120.8</v>
       </c>
-      <c r="D12" t="n">
+      <c r="E16" t="n">
         <v>118.2</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
+    <row r="17">
+      <c r="B17" s="4" t="n">
         <v>45622</v>
       </c>
-      <c r="B13" t="n">
+      <c r="C17" t="n">
         <v>145.2</v>
       </c>
-      <c r="C13" t="n">
+      <c r="D17" t="n">
         <v>125.1</v>
       </c>
-      <c r="D13" t="n">
+      <c r="E17" t="n">
         <v>121.5</v>
       </c>
     </row>
-    <row r="16">
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>Summary</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="F17" t="inlineStr">
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20">
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>Summary Returns</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="H21" s="3" t="inlineStr">
         <is>
           <t>Subject</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>Benchmark 1</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>Benchmark 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="F18" t="inlineStr">
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>Bench 1</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>Bench 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="G22" t="inlineStr">
         <is>
           <t>Cumulative Return</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="H22" t="inlineStr">
         <is>
           <t>45.2%</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t>25.1%</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="J22" t="inlineStr">
         <is>
           <t>21.5%</t>
         </is>

</xml_diff>